<commit_message>
Rebuild update_log.xlsx in one-row-per-file format with full history
</commit_message>
<xml_diff>
--- a/update_log.xlsx
+++ b/update_log.xlsx
@@ -425,144 +425,126 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Date &amp; Time (IST)</t>
+          <t>File Name</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>File Updated</t>
+          <t>Update 1</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Update Details</t>
+          <t>Update 2</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Update 3</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Update 4</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-08 10:11:00</t>
+          <t>hunter.py</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>hunter.py</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Fixed ValueError unpack crash in score_lead_ai fallback</t>
-        </is>
-      </c>
+          <t>2026-07-08 10:11 IST — Fixed ValueError unpack crash in score_lead_ai fallback (missing address N/A return value)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-08 10:32:00</t>
+          <t>gsheets_handler.py</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>gsheets_handler.py</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Added search offset cloud sync methods</t>
-        </is>
-      </c>
+          <t>2026-07-08 10:32 IST — Added load_search_offsets_from_cloud() and update_cloud_search_offset() for cross-device sync</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-07-08 10:40:00</t>
+          <t>dashboard.py</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>dashboard.py</t>
+          <t>2026-07-08 10:40 IST — Replaced Manual Outreach tab with RAM-optimized paginated CRM Hub + incremental CSV backup</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Replaced Manual Outreach tab with RAM-optimized CRM and added incremental backup</t>
+          <t>2026-07-08 10:48 IST — Fixed indentation SyntaxErrors from CRM script deployment</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-07-08 10:52 IST — Added WhatsApp Intent Radar Tracking (intelligence_opens.txt parser)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-07-08 10:55 IST — Injected auto-deduplicator on app startup (incremental_leads_backup.csv)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-08 10:52:00</t>
+          <t>plan_log.md</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>dashboard.py</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Added WhatsApp Intent Radar Tracking for intelligence_opens.txt</t>
-        </is>
-      </c>
+          <t>2026-07-08 10:52 IST — Created plan tracking log for all enhancements</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-07-08 10:52:00</t>
+          <t>log_update.py</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>plan_log.md</t>
+          <t>2026-07-08 10:58 IST — Created update log utility (single-file-per-row format)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Created plan tracking log</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-07-08 10:55:00</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>dashboard.py</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Injected auto-deduplicator on app startup</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-07-08 10:58 IST</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>log_update.py</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Created update log utility - auto-appends to update_log.xlsx and update_log.csv on every change</t>
-        </is>
-      </c>
+          <t>2026-07-08 11:01 IST — Rebuilt to one-row-per-file column format</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>